<commit_message>
Added EW 6 to 16
</commit_message>
<xml_diff>
--- a/SGP/SGP-ID-Bulletins.xlsx
+++ b/SGP/SGP-ID-Bulletins.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="213">
   <si>
     <t>source_file_name</t>
   </si>
@@ -202,6 +202,27 @@
     <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 1.pdf</t>
   </si>
   <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 10.pdf</t>
+  </si>
+  <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 11.pdf</t>
+  </si>
+  <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 12.pdf</t>
+  </si>
+  <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 13.pdf</t>
+  </si>
+  <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 14.pdf</t>
+  </si>
+  <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 15.pdf</t>
+  </si>
+  <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 16.pdf</t>
+  </si>
+  <si>
     <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 2.pdf</t>
   </si>
   <si>
@@ -214,6 +235,18 @@
     <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 5.pdf</t>
   </si>
   <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 6.pdf</t>
+  </si>
+  <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 7.pdf</t>
+  </si>
+  <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 8.pdf</t>
+  </si>
+  <si>
+    <t>c:/dev/covid-19-world-vaccinations/SGP/2026\Weekly Infectious Disease Bulletin EW 9.pdf</t>
+  </si>
+  <si>
     <t>4 - 10 May 2025</t>
   </si>
   <si>
@@ -373,6 +406,27 @@
     <t>4 - 10 Jan 2026</t>
   </si>
   <si>
+    <t>8 - 14 Mar 2026</t>
+  </si>
+  <si>
+    <t>15 - 21 Mar 2026</t>
+  </si>
+  <si>
+    <t>22 - 28 Mar 2026</t>
+  </si>
+  <si>
+    <t>29 Mar 2025 - 4 Apr 2026</t>
+  </si>
+  <si>
+    <t>5 - 11 Apr 2026</t>
+  </si>
+  <si>
+    <t>12 - 18 Apr 2026</t>
+  </si>
+  <si>
+    <t>19 - 25 Apr 2026</t>
+  </si>
+  <si>
     <t>11 - 17 Jan 2026</t>
   </si>
   <si>
@@ -385,6 +439,18 @@
     <t>1 - 7 Feb 2026</t>
   </si>
   <si>
+    <t>8 - 14 Feb 2026</t>
+  </si>
+  <si>
+    <t>15 - 21 Feb 2026</t>
+  </si>
+  <si>
+    <t>22 - 28 Feb 2026</t>
+  </si>
+  <si>
+    <t>1 - 7 Mar 2026</t>
+  </si>
+  <si>
     <t>10 May 2025</t>
   </si>
   <si>
@@ -544,6 +610,27 @@
     <t>10 Jan 2026</t>
   </si>
   <si>
+    <t>14 Mar 2026</t>
+  </si>
+  <si>
+    <t>21 Mar 2026</t>
+  </si>
+  <si>
+    <t>28 Mar 2026</t>
+  </si>
+  <si>
+    <t>4 Apr 2026</t>
+  </si>
+  <si>
+    <t>11 Apr 2026</t>
+  </si>
+  <si>
+    <t>18 Apr 2026</t>
+  </si>
+  <si>
+    <t>25 Apr 2026</t>
+  </si>
+  <si>
     <t>17 Jan 2026</t>
   </si>
   <si>
@@ -554,6 +641,18 @@
   </si>
   <si>
     <t>7 Feb 2026</t>
+  </si>
+  <si>
+    <t>14 Feb 2026</t>
+  </si>
+  <si>
+    <t>21 Feb 2026</t>
+  </si>
+  <si>
+    <t>28 Feb 2026</t>
+  </si>
+  <si>
+    <t>7 Mar 2026</t>
   </si>
 </sst>
 </file>
@@ -911,7 +1010,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -954,10 +1053,10 @@
         <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="E2" t="s">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="F2">
         <v>2711</v>
@@ -986,10 +1085,10 @@
         <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="E3" t="s">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="F3">
         <v>2636</v>
@@ -1018,10 +1117,10 @@
         <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="F4">
         <v>2338</v>
@@ -1050,10 +1149,10 @@
         <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E5" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="F5">
         <v>2154</v>
@@ -1082,10 +1181,10 @@
         <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E6" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="F6">
         <v>1996</v>
@@ -1114,10 +1213,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="E7" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -1146,10 +1245,10 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="E8" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="F8">
         <v>2714</v>
@@ -1178,10 +1277,10 @@
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="E9" t="s">
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="F9">
         <v>2866</v>
@@ -1210,10 +1309,10 @@
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="E10" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
       <c r="F10">
         <v>3045</v>
@@ -1242,10 +1341,10 @@
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="E11" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="F11">
         <v>3392</v>
@@ -1274,10 +1373,10 @@
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="E12" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="F12">
         <v>3046</v>
@@ -1306,10 +1405,10 @@
         <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="E13" t="s">
-        <v>134</v>
+        <v>156</v>
       </c>
       <c r="F13">
         <v>2542</v>
@@ -1338,10 +1437,10 @@
         <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="E14" t="s">
-        <v>135</v>
+        <v>157</v>
       </c>
       <c r="F14">
         <v>2431</v>
@@ -1370,10 +1469,10 @@
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="E15" t="s">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="F15">
         <v>2179</v>
@@ -1402,10 +1501,10 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="F16">
         <v>2424</v>
@@ -1434,10 +1533,10 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="E17" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="F17">
         <v>2471</v>
@@ -1466,10 +1565,10 @@
         <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E18" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="F18">
         <v>2632</v>
@@ -1498,10 +1597,10 @@
         <v>16</v>
       </c>
       <c r="D19" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="E19" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="F19">
         <v>2749</v>
@@ -1530,10 +1629,10 @@
         <v>17</v>
       </c>
       <c r="D20" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="E20" t="s">
-        <v>141</v>
+        <v>163</v>
       </c>
       <c r="F20">
         <v>2781</v>
@@ -1562,10 +1661,10 @@
         <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="E21" t="s">
-        <v>142</v>
+        <v>164</v>
       </c>
       <c r="F21">
         <v>2906</v>
@@ -1594,10 +1693,10 @@
         <v>20</v>
       </c>
       <c r="D22" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="E22" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="F22">
         <v>2828</v>
@@ -1626,10 +1725,10 @@
         <v>21</v>
       </c>
       <c r="D23" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="E23" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="F23">
         <v>2856</v>
@@ -1658,10 +1757,10 @@
         <v>26</v>
       </c>
       <c r="D24" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="E24" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="F24">
         <v>2018</v>
@@ -1690,10 +1789,10 @@
         <v>27</v>
       </c>
       <c r="D25" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E25" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="F25">
         <v>2147</v>
@@ -1722,10 +1821,10 @@
         <v>28</v>
       </c>
       <c r="D26" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="E26" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="F26">
         <v>2148</v>
@@ -1754,10 +1853,10 @@
         <v>29</v>
       </c>
       <c r="D27" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="E27" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="F27">
         <v>2282</v>
@@ -1786,10 +1885,10 @@
         <v>31</v>
       </c>
       <c r="D28" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="E28" t="s">
-        <v>149</v>
+        <v>171</v>
       </c>
       <c r="F28">
         <v>2298</v>
@@ -1818,10 +1917,10 @@
         <v>33</v>
       </c>
       <c r="D29" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="E29" t="s">
-        <v>150</v>
+        <v>172</v>
       </c>
       <c r="F29">
         <v>2353</v>
@@ -1850,10 +1949,10 @@
         <v>34</v>
       </c>
       <c r="D30" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="E30" t="s">
-        <v>151</v>
+        <v>173</v>
       </c>
       <c r="F30">
         <v>2501</v>
@@ -1882,10 +1981,10 @@
         <v>35</v>
       </c>
       <c r="D31" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="E31" t="s">
-        <v>152</v>
+        <v>174</v>
       </c>
       <c r="F31">
         <v>2553</v>
@@ -1914,10 +2013,10 @@
         <v>36</v>
       </c>
       <c r="D32" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E32" t="s">
-        <v>153</v>
+        <v>175</v>
       </c>
       <c r="F32">
         <v>2520</v>
@@ -1946,10 +2045,10 @@
         <v>37</v>
       </c>
       <c r="D33" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="E33" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
       <c r="F33">
         <v>2498</v>
@@ -1978,10 +2077,10 @@
         <v>38</v>
       </c>
       <c r="D34" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="E34" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="F34">
         <v>2809</v>
@@ -2010,10 +2109,10 @@
         <v>39</v>
       </c>
       <c r="D35" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="E35" t="s">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="F35">
         <v>2748</v>
@@ -2042,10 +2141,10 @@
         <v>40</v>
       </c>
       <c r="D36" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="E36" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="F36">
         <v>2646</v>
@@ -2074,10 +2173,10 @@
         <v>41</v>
       </c>
       <c r="D37" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="E37" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="F37">
         <v>2715</v>
@@ -2106,10 +2205,10 @@
         <v>42</v>
       </c>
       <c r="D38" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="E38" t="s">
-        <v>159</v>
+        <v>181</v>
       </c>
       <c r="F38">
         <v>2776</v>
@@ -2138,10 +2237,10 @@
         <v>44</v>
       </c>
       <c r="D39" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="E39" t="s">
-        <v>160</v>
+        <v>182</v>
       </c>
       <c r="F39">
         <v>2592</v>
@@ -2170,10 +2269,10 @@
         <v>45</v>
       </c>
       <c r="D40" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="E40" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="F40">
         <v>2487</v>
@@ -2202,10 +2301,10 @@
         <v>46</v>
       </c>
       <c r="D41" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="E41" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
       <c r="F41">
         <v>2445</v>
@@ -2234,10 +2333,10 @@
         <v>47</v>
       </c>
       <c r="D42" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="E42" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
       <c r="F42">
         <v>2443</v>
@@ -2266,10 +2365,10 @@
         <v>48</v>
       </c>
       <c r="D43" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="E43" t="s">
-        <v>164</v>
+        <v>186</v>
       </c>
       <c r="F43">
         <v>2450</v>
@@ -2298,10 +2397,10 @@
         <v>49</v>
       </c>
       <c r="D44" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="E44" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
       <c r="F44">
         <v>2452</v>
@@ -2330,10 +2429,10 @@
         <v>50</v>
       </c>
       <c r="D45" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="E45" t="s">
-        <v>166</v>
+        <v>188</v>
       </c>
       <c r="F45">
         <v>2523</v>
@@ -2362,10 +2461,10 @@
         <v>51</v>
       </c>
       <c r="D46" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="E46" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
       <c r="F46">
         <v>2452</v>
@@ -2394,10 +2493,10 @@
         <v>52</v>
       </c>
       <c r="D47" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="E47" t="s">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="F47">
         <v>2735</v>
@@ -2426,10 +2525,10 @@
         <v>53</v>
       </c>
       <c r="D48" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="E48" t="s">
-        <v>169</v>
+        <v>191</v>
       </c>
       <c r="F48">
         <v>2832</v>
@@ -2458,10 +2557,10 @@
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="E49" t="s">
-        <v>170</v>
+        <v>192</v>
       </c>
       <c r="F49">
         <v>2617</v>
@@ -2490,10 +2589,10 @@
         <v>32</v>
       </c>
       <c r="D50" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="E50" t="s">
-        <v>171</v>
+        <v>193</v>
       </c>
       <c r="F50">
         <v>2274</v>
@@ -2522,10 +2621,10 @@
         <v>6</v>
       </c>
       <c r="D51" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="E51" t="s">
-        <v>172</v>
+        <v>194</v>
       </c>
       <c r="F51">
         <v>3381</v>
@@ -2554,10 +2653,10 @@
         <v>8</v>
       </c>
       <c r="D52" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="E52" t="s">
-        <v>173</v>
+        <v>195</v>
       </c>
       <c r="F52">
         <v>2749</v>
@@ -2586,10 +2685,10 @@
         <v>30</v>
       </c>
       <c r="D53" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="E53" t="s">
-        <v>174</v>
+        <v>196</v>
       </c>
       <c r="F53">
         <v>2304</v>
@@ -2618,10 +2717,10 @@
         <v>1</v>
       </c>
       <c r="D54" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="E54" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="F54">
         <v>2857</v>
@@ -2647,16 +2746,16 @@
         <v>62</v>
       </c>
       <c r="C55">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D55" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="E55" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="F55">
-        <v>2938</v>
+        <v>0</v>
       </c>
       <c r="G55">
         <v>0</v>
@@ -2665,10 +2764,10 @@
         <v>0</v>
       </c>
       <c r="I55">
-        <v>260</v>
+        <v>305</v>
       </c>
       <c r="J55">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -2679,28 +2778,28 @@
         <v>63</v>
       </c>
       <c r="C56">
+        <v>11</v>
+      </c>
+      <c r="D56" t="s">
+        <v>131</v>
+      </c>
+      <c r="E56" t="s">
+        <v>199</v>
+      </c>
+      <c r="F56">
+        <v>2377</v>
+      </c>
+      <c r="G56">
+        <v>0</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56">
+        <v>221</v>
+      </c>
+      <c r="J56">
         <v>3</v>
-      </c>
-      <c r="D56" t="s">
-        <v>120</v>
-      </c>
-      <c r="E56" t="s">
-        <v>177</v>
-      </c>
-      <c r="F56">
-        <v>3093</v>
-      </c>
-      <c r="G56">
-        <v>0</v>
-      </c>
-      <c r="H56">
-        <v>0</v>
-      </c>
-      <c r="I56">
-        <v>281</v>
-      </c>
-      <c r="J56">
-        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -2711,16 +2810,16 @@
         <v>64</v>
       </c>
       <c r="C57">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D57" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="E57" t="s">
-        <v>178</v>
+        <v>200</v>
       </c>
       <c r="F57">
-        <v>3017</v>
+        <v>2500</v>
       </c>
       <c r="G57">
         <v>0</v>
@@ -2729,10 +2828,10 @@
         <v>0</v>
       </c>
       <c r="I57">
-        <v>0</v>
+        <v>233</v>
       </c>
       <c r="J57">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -2743,28 +2842,380 @@
         <v>65</v>
       </c>
       <c r="C58">
+        <v>13</v>
+      </c>
+      <c r="D58" t="s">
+        <v>133</v>
+      </c>
+      <c r="E58" t="s">
+        <v>201</v>
+      </c>
+      <c r="F58">
+        <v>2512</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58">
+        <v>169</v>
+      </c>
+      <c r="J58">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10">
+      <c r="A59" s="1">
+        <v>57</v>
+      </c>
+      <c r="B59" t="s">
+        <v>66</v>
+      </c>
+      <c r="C59">
+        <v>14</v>
+      </c>
+      <c r="D59" t="s">
+        <v>134</v>
+      </c>
+      <c r="E59" t="s">
+        <v>202</v>
+      </c>
+      <c r="F59">
+        <v>2512</v>
+      </c>
+      <c r="G59">
+        <v>0</v>
+      </c>
+      <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59">
+        <v>216</v>
+      </c>
+      <c r="J59">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10">
+      <c r="A60" s="1">
+        <v>58</v>
+      </c>
+      <c r="B60" t="s">
+        <v>67</v>
+      </c>
+      <c r="C60">
+        <v>15</v>
+      </c>
+      <c r="D60" t="s">
+        <v>135</v>
+      </c>
+      <c r="E60" t="s">
+        <v>203</v>
+      </c>
+      <c r="F60">
+        <v>2531</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60">
+        <v>0</v>
+      </c>
+      <c r="I60">
+        <v>231</v>
+      </c>
+      <c r="J60">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
+      <c r="A61" s="1">
+        <v>59</v>
+      </c>
+      <c r="B61" t="s">
+        <v>68</v>
+      </c>
+      <c r="C61">
+        <v>16</v>
+      </c>
+      <c r="D61" t="s">
+        <v>136</v>
+      </c>
+      <c r="E61" t="s">
+        <v>204</v>
+      </c>
+      <c r="F61">
+        <v>2590</v>
+      </c>
+      <c r="G61">
         <v>5</v>
       </c>
-      <c r="D58" t="s">
-        <v>122</v>
-      </c>
-      <c r="E58" t="s">
-        <v>179</v>
-      </c>
-      <c r="F58">
+      <c r="H61">
+        <v>0</v>
+      </c>
+      <c r="I61">
+        <v>229</v>
+      </c>
+      <c r="J61">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
+      <c r="A62" s="1">
+        <v>60</v>
+      </c>
+      <c r="B62" t="s">
+        <v>69</v>
+      </c>
+      <c r="C62">
+        <v>2</v>
+      </c>
+      <c r="D62" t="s">
+        <v>137</v>
+      </c>
+      <c r="E62" t="s">
+        <v>205</v>
+      </c>
+      <c r="F62">
+        <v>2938</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62">
+        <v>0</v>
+      </c>
+      <c r="I62">
+        <v>260</v>
+      </c>
+      <c r="J62">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10">
+      <c r="A63" s="1">
+        <v>61</v>
+      </c>
+      <c r="B63" t="s">
+        <v>70</v>
+      </c>
+      <c r="C63">
+        <v>3</v>
+      </c>
+      <c r="D63" t="s">
+        <v>138</v>
+      </c>
+      <c r="E63" t="s">
+        <v>206</v>
+      </c>
+      <c r="F63">
+        <v>3093</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63">
+        <v>281</v>
+      </c>
+      <c r="J63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10">
+      <c r="A64" s="1">
+        <v>62</v>
+      </c>
+      <c r="B64" t="s">
+        <v>71</v>
+      </c>
+      <c r="C64">
+        <v>4</v>
+      </c>
+      <c r="D64" t="s">
+        <v>139</v>
+      </c>
+      <c r="E64" t="s">
+        <v>207</v>
+      </c>
+      <c r="F64">
+        <v>3017</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64">
+        <v>0</v>
+      </c>
+      <c r="J64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10">
+      <c r="A65" s="1">
+        <v>63</v>
+      </c>
+      <c r="B65" t="s">
+        <v>72</v>
+      </c>
+      <c r="C65">
+        <v>5</v>
+      </c>
+      <c r="D65" t="s">
+        <v>140</v>
+      </c>
+      <c r="E65" t="s">
+        <v>208</v>
+      </c>
+      <c r="F65">
         <v>2992</v>
       </c>
-      <c r="G58">
-        <v>0</v>
-      </c>
-      <c r="H58">
-        <v>0</v>
-      </c>
-      <c r="I58">
-        <v>0</v>
-      </c>
-      <c r="J58">
-        <v>0</v>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65">
+        <v>0</v>
+      </c>
+      <c r="J65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10">
+      <c r="A66" s="1">
+        <v>64</v>
+      </c>
+      <c r="B66" t="s">
+        <v>73</v>
+      </c>
+      <c r="C66">
+        <v>6</v>
+      </c>
+      <c r="D66" t="s">
+        <v>141</v>
+      </c>
+      <c r="E66" t="s">
+        <v>209</v>
+      </c>
+      <c r="F66">
+        <v>2835</v>
+      </c>
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66">
+        <v>0</v>
+      </c>
+      <c r="I66">
+        <v>311</v>
+      </c>
+      <c r="J66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10">
+      <c r="A67" s="1">
+        <v>65</v>
+      </c>
+      <c r="B67" t="s">
+        <v>74</v>
+      </c>
+      <c r="C67">
+        <v>7</v>
+      </c>
+      <c r="D67" t="s">
+        <v>142</v>
+      </c>
+      <c r="E67" t="s">
+        <v>210</v>
+      </c>
+      <c r="F67">
+        <v>3039</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <v>0</v>
+      </c>
+      <c r="I67">
+        <v>0</v>
+      </c>
+      <c r="J67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10">
+      <c r="A68" s="1">
+        <v>66</v>
+      </c>
+      <c r="B68" t="s">
+        <v>75</v>
+      </c>
+      <c r="C68">
+        <v>8</v>
+      </c>
+      <c r="D68" t="s">
+        <v>143</v>
+      </c>
+      <c r="E68" t="s">
+        <v>211</v>
+      </c>
+      <c r="F68">
+        <v>2801</v>
+      </c>
+      <c r="G68">
+        <v>0</v>
+      </c>
+      <c r="H68">
+        <v>0</v>
+      </c>
+      <c r="I68">
+        <v>309</v>
+      </c>
+      <c r="J68">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10">
+      <c r="A69" s="1">
+        <v>67</v>
+      </c>
+      <c r="B69" t="s">
+        <v>76</v>
+      </c>
+      <c r="C69">
+        <v>9</v>
+      </c>
+      <c r="D69" t="s">
+        <v>144</v>
+      </c>
+      <c r="E69" t="s">
+        <v>212</v>
+      </c>
+      <c r="F69">
+        <v>2760</v>
+      </c>
+      <c r="G69">
+        <v>0</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <v>276</v>
+      </c>
+      <c r="J69">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>